<commit_message>
Version2 review 1 report
</commit_message>
<xml_diff>
--- a/review_test_cases/10_special_case/review2case.xlsx
+++ b/review_test_cases/10_special_case/review2case.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HydrogenRb\HydrogenRb\Work\tech\Agent\8_14\review_test_cases\10_special_case\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56E38D6D-61E5-494A-986A-4FA9DB07CCBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC5B1E6-17D5-4622-8671-EE58B8E3DEA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="集成" sheetId="1" r:id="rId1"/>
     <sheet name="RISCV_TOP" sheetId="2" r:id="rId2"/>
     <sheet name="RISCV_CORE_TEST" sheetId="3" r:id="rId3"/>
     <sheet name="MEM_PHY" sheetId="4" r:id="rId4"/>
+    <sheet name="mem_dat" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="85">
   <si>
     <t>分类</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -298,6 +299,73 @@
   </si>
   <si>
     <t>`APB_1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>array_2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>`LANE_NUM*`Test_size</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>5*100</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>范围是{11,12,13}</t>
+  </si>
+  <si>
+    <t>范围是{11,12,13}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>大位宽输入输出</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>bus_in</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BUS_IN</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>dyadic_bus_out_{{z}}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>z的范围是{dat,req,rsp}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BUS_OUT_{{z}}*DW</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>范围是{{32,32,64}}*8</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MEM_DAT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BUS_OUT_{{z}}*DW*BUS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>范围是{{32,32,64}}*8*5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>bus_in[i]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>dyadic_bus_out_{{z}}[i]</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -626,15 +694,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y22"/>
+  <dimension ref="A1:AA25"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="3" max="3" width="9.33203125" customWidth="1"/>
     <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="10" max="10" width="10.1328125" customWidth="1"/>
+    <col min="12" max="12" width="10.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.4">
       <c r="B1" s="1" t="s">
         <v>28</v>
       </c>
@@ -647,28 +715,32 @@
         <v>30</v>
       </c>
       <c r="G1" s="1"/>
-      <c r="J1" s="1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1" s="1"/>
+      <c r="L1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1"/>
+      <c r="N1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="M1" s="1"/>
-      <c r="P1" s="1" t="s">
+      <c r="O1" s="1"/>
+      <c r="R1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="Q1" s="1"/>
-      <c r="T1" s="1" t="s">
+      <c r="S1" s="1"/>
+      <c r="V1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="U1" s="1"/>
-      <c r="X1" s="1" t="s">
+      <c r="W1" s="1"/>
+      <c r="Z1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="Y1" s="1"/>
-    </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="AA1" s="1"/>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -690,14 +762,8 @@
       <c r="G2" t="s">
         <v>2</v>
       </c>
-      <c r="I2" t="s">
+      <c r="K2" t="s">
         <v>0</v>
-      </c>
-      <c r="J2" t="s">
-        <v>1</v>
-      </c>
-      <c r="K2" t="s">
-        <v>2</v>
       </c>
       <c r="L2" t="s">
         <v>1</v>
@@ -705,35 +771,41 @@
       <c r="M2" t="s">
         <v>2</v>
       </c>
+      <c r="N2" t="s">
+        <v>1</v>
+      </c>
       <c r="O2" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q2" t="s">
         <v>0</v>
       </c>
-      <c r="P2" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
+        <v>1</v>
+      </c>
+      <c r="S2" t="s">
         <v>2</v>
       </c>
-      <c r="S2" t="s">
+      <c r="U2" t="s">
         <v>0</v>
       </c>
-      <c r="T2" t="s">
-        <v>1</v>
-      </c>
-      <c r="U2" t="s">
+      <c r="V2" t="s">
+        <v>1</v>
+      </c>
+      <c r="W2" t="s">
         <v>2</v>
       </c>
-      <c r="W2" t="s">
+      <c r="Y2" t="s">
         <v>0</v>
       </c>
-      <c r="X2" t="s">
-        <v>1</v>
-      </c>
-      <c r="Y2" t="s">
+      <c r="Z2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AA2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -755,50 +827,50 @@
       <c r="G3" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="J3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K3" t="s">
-        <v>5</v>
       </c>
       <c r="L3" t="s">
         <v>14</v>
       </c>
       <c r="M3" t="s">
-        <v>20</v>
-      </c>
-      <c r="O3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="N3" t="s">
+        <v>14</v>
+      </c>
+      <c r="O3" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="P3" t="s">
+      <c r="R3" t="s">
         <v>21</v>
       </c>
-      <c r="Q3" t="s">
-        <v>5</v>
-      </c>
-      <c r="S3" s="1" t="s">
+      <c r="S3" t="s">
+        <v>5</v>
+      </c>
+      <c r="U3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="T3" t="s">
+      <c r="V3" t="s">
         <v>21</v>
       </c>
-      <c r="U3" t="s">
-        <v>5</v>
-      </c>
-      <c r="W3" s="1" t="s">
+      <c r="W3" t="s">
+        <v>5</v>
+      </c>
+      <c r="Y3" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="X3" t="s">
+      <c r="Z3" t="s">
         <v>21</v>
       </c>
-      <c r="Y3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="AA3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.4">
       <c r="A4" s="1"/>
       <c r="B4" t="s">
         <v>38</v>
@@ -818,78 +890,78 @@
       <c r="G4" t="s">
         <v>5</v>
       </c>
-      <c r="I4" s="1"/>
-      <c r="J4" t="s">
-        <v>15</v>
-      </c>
-      <c r="K4" t="s">
-        <v>5</v>
-      </c>
+      <c r="K4" s="1"/>
       <c r="L4" t="s">
         <v>15</v>
       </c>
       <c r="M4" t="s">
-        <v>20</v>
-      </c>
-      <c r="O4" s="1"/>
-      <c r="P4" t="s">
+        <v>5</v>
+      </c>
+      <c r="N4" t="s">
+        <v>15</v>
+      </c>
+      <c r="O4" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q4" s="1"/>
+      <c r="R4" t="s">
         <v>23</v>
       </c>
-      <c r="Q4" t="s">
-        <v>5</v>
-      </c>
-      <c r="S4" s="1"/>
-      <c r="T4" t="s">
+      <c r="S4" t="s">
+        <v>5</v>
+      </c>
+      <c r="U4" s="1"/>
+      <c r="V4" t="s">
         <v>23</v>
       </c>
-      <c r="U4" t="s">
-        <v>5</v>
-      </c>
-      <c r="W4" s="1"/>
-      <c r="X4" t="s">
+      <c r="W4" t="s">
+        <v>5</v>
+      </c>
+      <c r="Y4" s="1"/>
+      <c r="Z4" t="s">
         <v>23</v>
       </c>
-      <c r="Y4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="I5" s="1"/>
-      <c r="J5" t="s">
-        <v>16</v>
-      </c>
-      <c r="K5" t="s">
-        <v>20</v>
-      </c>
+      <c r="AA4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.4">
+      <c r="K5" s="1"/>
       <c r="L5" t="s">
         <v>16</v>
       </c>
       <c r="M5" t="s">
-        <v>5</v>
-      </c>
-      <c r="O5" s="1"/>
-      <c r="P5" t="s">
+        <v>20</v>
+      </c>
+      <c r="N5" t="s">
+        <v>16</v>
+      </c>
+      <c r="O5" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q5" s="1"/>
+      <c r="R5" t="s">
         <v>24</v>
       </c>
-      <c r="Q5" t="s">
-        <v>20</v>
-      </c>
-      <c r="S5" s="1"/>
-      <c r="T5" t="s">
+      <c r="S5" t="s">
+        <v>20</v>
+      </c>
+      <c r="U5" s="1"/>
+      <c r="V5" t="s">
         <v>24</v>
       </c>
-      <c r="U5" t="s">
-        <v>20</v>
-      </c>
-      <c r="W5" s="1"/>
-      <c r="X5" t="s">
+      <c r="W5" t="s">
+        <v>20</v>
+      </c>
+      <c r="Y5" s="1"/>
+      <c r="Z5" t="s">
         <v>24</v>
       </c>
-      <c r="Y5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="AA5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -905,42 +977,42 @@
       <c r="G6" t="s">
         <v>5</v>
       </c>
-      <c r="I6" s="1"/>
-      <c r="J6" t="s">
-        <v>17</v>
-      </c>
-      <c r="K6" t="s">
-        <v>20</v>
-      </c>
+      <c r="K6" s="1"/>
       <c r="L6" t="s">
         <v>17</v>
       </c>
       <c r="M6" t="s">
-        <v>5</v>
-      </c>
-      <c r="O6" s="1"/>
-      <c r="P6" t="s">
+        <v>20</v>
+      </c>
+      <c r="N6" t="s">
+        <v>17</v>
+      </c>
+      <c r="O6" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q6" s="1"/>
+      <c r="R6" t="s">
         <v>25</v>
       </c>
-      <c r="Q6" t="s">
-        <v>20</v>
-      </c>
-      <c r="S6" s="1"/>
-      <c r="T6" t="s">
+      <c r="S6" t="s">
+        <v>20</v>
+      </c>
+      <c r="U6" s="1"/>
+      <c r="V6" t="s">
         <v>25</v>
       </c>
-      <c r="U6" t="s">
-        <v>20</v>
-      </c>
-      <c r="W6" s="1"/>
-      <c r="X6" t="s">
+      <c r="W6" t="s">
+        <v>20</v>
+      </c>
+      <c r="Y6" s="1"/>
+      <c r="Z6" t="s">
         <v>25</v>
       </c>
-      <c r="Y6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="AA6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" x14ac:dyDescent="0.4">
       <c r="A7" s="1"/>
       <c r="B7" t="s">
         <v>8</v>
@@ -954,42 +1026,42 @@
       <c r="G7" t="s">
         <v>5</v>
       </c>
-      <c r="I7" s="1"/>
-      <c r="J7" t="s">
-        <v>18</v>
-      </c>
-      <c r="K7" t="s">
-        <v>20</v>
-      </c>
+      <c r="K7" s="1"/>
       <c r="L7" t="s">
         <v>18</v>
       </c>
       <c r="M7" t="s">
-        <v>5</v>
-      </c>
-      <c r="O7" s="1"/>
-      <c r="P7" t="s">
+        <v>20</v>
+      </c>
+      <c r="N7" t="s">
+        <v>18</v>
+      </c>
+      <c r="O7" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q7" s="1"/>
+      <c r="R7" t="s">
         <v>26</v>
       </c>
-      <c r="Q7" t="s">
-        <v>20</v>
-      </c>
-      <c r="S7" s="1"/>
-      <c r="T7" t="s">
+      <c r="S7" t="s">
+        <v>20</v>
+      </c>
+      <c r="U7" s="1"/>
+      <c r="V7" t="s">
         <v>26</v>
       </c>
-      <c r="U7" t="s">
-        <v>20</v>
-      </c>
-      <c r="W7" s="1"/>
-      <c r="X7" t="s">
+      <c r="W7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Y7" s="1"/>
+      <c r="Z7" t="s">
         <v>26</v>
       </c>
-      <c r="Y7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="AA7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.4">
       <c r="A8" s="1"/>
       <c r="B8" t="s">
         <v>9</v>
@@ -1009,42 +1081,42 @@
       <c r="G8" t="s">
         <v>5</v>
       </c>
-      <c r="I8" s="1"/>
-      <c r="J8" t="s">
-        <v>19</v>
-      </c>
-      <c r="K8" t="s">
-        <v>20</v>
-      </c>
+      <c r="K8" s="1"/>
       <c r="L8" t="s">
         <v>19</v>
       </c>
       <c r="M8" t="s">
-        <v>5</v>
-      </c>
-      <c r="O8" s="1"/>
-      <c r="P8" t="s">
+        <v>20</v>
+      </c>
+      <c r="N8" t="s">
+        <v>19</v>
+      </c>
+      <c r="O8" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q8" s="1"/>
+      <c r="R8" t="s">
         <v>26</v>
       </c>
-      <c r="Q8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S8" s="1"/>
-      <c r="T8" t="s">
+      <c r="S8" t="s">
+        <v>20</v>
+      </c>
+      <c r="U8" s="1"/>
+      <c r="V8" t="s">
         <v>26</v>
       </c>
-      <c r="U8" t="s">
-        <v>20</v>
-      </c>
-      <c r="W8" s="1"/>
-      <c r="X8" t="s">
+      <c r="W8" t="s">
+        <v>20</v>
+      </c>
+      <c r="Y8" s="1"/>
+      <c r="Z8" t="s">
         <v>26</v>
       </c>
-      <c r="Y8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="AA8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" x14ac:dyDescent="0.4">
       <c r="A9" s="1"/>
       <c r="B9" t="s">
         <v>10</v>
@@ -1064,23 +1136,23 @@
       <c r="G9" t="s">
         <v>5</v>
       </c>
-      <c r="I9" t="s">
+      <c r="K9" t="s">
         <v>56</v>
-      </c>
-      <c r="J9" t="s">
-        <v>57</v>
-      </c>
-      <c r="K9" t="s">
-        <v>20</v>
       </c>
       <c r="L9" t="s">
         <v>57</v>
       </c>
       <c r="M9" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+      <c r="N9" t="s">
+        <v>57</v>
+      </c>
+      <c r="O9" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.4">
       <c r="A10" s="1"/>
       <c r="B10" t="s">
         <v>11</v>
@@ -1089,7 +1161,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -1112,7 +1184,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
         <v>47</v>
       </c>
@@ -1135,7 +1207,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.4">
       <c r="A15" s="1"/>
       <c r="B15" t="s">
         <v>45</v>
@@ -1156,7 +1228,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.4">
       <c r="A16" s="1"/>
       <c r="B16" t="s">
         <v>46</v>
@@ -1177,7 +1249,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>52</v>
       </c>
@@ -1194,7 +1266,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A20" s="1" t="s">
         <v>61</v>
       </c>
@@ -1211,7 +1283,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A21" s="1"/>
       <c r="B21" t="s">
         <v>63</v>
@@ -1226,7 +1298,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A22" s="1"/>
       <c r="B22" t="s">
         <v>64</v>
@@ -1241,21 +1313,55 @@
         <v>20</v>
       </c>
     </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A24" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B24" t="s">
+        <v>83</v>
+      </c>
+      <c r="C24" t="s">
+        <v>5</v>
+      </c>
+      <c r="H24" t="s">
+        <v>74</v>
+      </c>
+      <c r="I24" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A25" s="1"/>
+      <c r="B25" t="s">
+        <v>84</v>
+      </c>
+      <c r="C25" t="s">
+        <v>20</v>
+      </c>
+      <c r="H25" t="s">
+        <v>76</v>
+      </c>
+      <c r="I25" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="18">
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="H1:I1"/>
     <mergeCell ref="A20:A22"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="O3:O8"/>
-    <mergeCell ref="T1:U1"/>
-    <mergeCell ref="S3:S8"/>
-    <mergeCell ref="X1:Y1"/>
-    <mergeCell ref="W3:W8"/>
+    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="Q3:Q8"/>
+    <mergeCell ref="V1:W1"/>
+    <mergeCell ref="U3:U8"/>
+    <mergeCell ref="Z1:AA1"/>
+    <mergeCell ref="Y3:Y8"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="A6:A10"/>
     <mergeCell ref="A14:A16"/>
-    <mergeCell ref="J1:K1"/>
     <mergeCell ref="L1:M1"/>
-    <mergeCell ref="I3:I8"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="K3:K8"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="F1:G1"/>
@@ -1267,8 +1373,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{202D62A6-CB45-4A21-B036-6EE2427F8DDC}">
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="4" max="4" width="23.06640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.4">
       <c r="B1" t="s">
@@ -1374,7 +1483,7 @@
         <v>9</v>
       </c>
       <c r="E8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F8" t="s">
         <v>5</v>
@@ -1563,6 +1672,9 @@
       <c r="D27" t="s">
         <v>49</v>
       </c>
+      <c r="E27" t="s">
+        <v>71</v>
+      </c>
       <c r="F27" t="s">
         <v>5</v>
       </c>
@@ -1588,8 +1700,44 @@
         <v>20</v>
       </c>
     </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A31" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B31" t="s">
+        <v>74</v>
+      </c>
+      <c r="D31" t="s">
+        <v>75</v>
+      </c>
+      <c r="E31">
+        <v>5</v>
+      </c>
+      <c r="F31" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A32" s="1"/>
+      <c r="B32" t="s">
+        <v>76</v>
+      </c>
+      <c r="D32" t="s">
+        <v>81</v>
+      </c>
+      <c r="E32" t="s">
+        <v>82</v>
+      </c>
+      <c r="F32" t="s">
+        <v>20</v>
+      </c>
+      <c r="I32" t="s">
+        <v>77</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="A31:A32"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="A6:A10"/>
     <mergeCell ref="A14:A19"/>
@@ -1603,8 +1751,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1F3E398-7E0A-4C3A-A273-DA12B1D3ED24}">
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="4" max="4" width="37.06640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.4">
       <c r="B1" t="s">
@@ -1925,7 +2076,7 @@
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.4">
-      <c r="A31" t="s">
+      <c r="A31" s="1" t="s">
         <v>56</v>
       </c>
       <c r="B31" t="s">
@@ -1941,49 +2092,78 @@
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.4">
-      <c r="A33" s="1" t="s">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A32" s="1"/>
+      <c r="B32" t="s">
+        <v>68</v>
+      </c>
+      <c r="D32" t="s">
+        <v>69</v>
+      </c>
+      <c r="E32" t="s">
+        <v>70</v>
+      </c>
+      <c r="F32" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A34" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B34" t="s">
         <v>62</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D34" t="s">
         <v>49</v>
       </c>
-      <c r="F33" t="s">
-        <v>5</v>
-      </c>
-      <c r="I33" t="s">
+      <c r="E34" t="s">
+        <v>72</v>
+      </c>
+      <c r="F34" t="s">
+        <v>5</v>
+      </c>
+      <c r="I34" t="s">
         <v>65</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.4">
-      <c r="A34" s="1"/>
-      <c r="B34" t="s">
-        <v>63</v>
-      </c>
-      <c r="F34" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A35" s="1"/>
       <c r="B35" t="s">
+        <v>63</v>
+      </c>
+      <c r="F35" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A36" s="1"/>
+      <c r="B36" t="s">
         <v>64</v>
       </c>
-      <c r="F35" t="s">
-        <v>20</v>
-      </c>
+      <c r="F36" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A38" s="1"/>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A39" s="1"/>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A40" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A33:A35"/>
+  <mergeCells count="8">
+    <mergeCell ref="A38:A40"/>
+    <mergeCell ref="A34:A36"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="A11:A16"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A18:A23"/>
     <mergeCell ref="A25:A27"/>
+    <mergeCell ref="A31:A32"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2378,4 +2558,84 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F31BFC09-6C83-41CA-81B5-6FE33A0231A4}">
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="B1" t="s">
+        <v>80</v>
+      </c>
+      <c r="H1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A3" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A4" s="1"/>
+      <c r="B4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E4" t="s">
+        <v>79</v>
+      </c>
+      <c r="F4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:A4"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>